<commit_message>
Sign outreach emails as Gabriel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAWtfhwVbimX9RKznBAhMh
</commit_message>
<xml_diff>
--- a/Australia_Trading_Bot_Prospects_200.xlsx
+++ b/Australia_Trading_Bot_Prospects_200.xlsx
@@ -660,7 +660,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. On Bitaroo that usually means small, auditable DCA or limit-order bots that only use trade permissions.
 Is this something your users ask you about?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -701,7 +701,7 @@
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. State/city not verified this session (search budget exhausted); fill in before use. QC: state '' not an Australian state/territory; email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. State/city not verified this session (search budget exhausted); fill in before use. QC: state '' not an Australian state/territory; email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
 For a fund like yours that usually means exchange API scripts for rebalancing and execution, plus a simple dashboard that reconciles positions across venues.
 Is any part of your trading workflow still handled by hand that you would like automated?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -832,7 +832,7 @@
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact apollocrypto.com page carrying the email not isolated (funds/wholesale/home pages returned). Sydney location from general knowledge, not re-verified this session. Strategy is largely discretionary/fundamental, not purely systematic. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact apollocrypto.com page carrying the email not isolated (funds/wholesale/home pages returned). Sydney location from general knowledge, not re-verified this session. Strategy is largely discretionary/fundamental, not purely systematic. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Blueberry that usually means Pine-to-MQL conversions and EA builds your support team can point clients towards.
 Would a developer referral like that be helpful for your clients?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -955,7 +955,7 @@
       <c r="W4" s="3" t="n"/>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For BullCharts that might mean a small bridge that takes scan results and forwards them to a broker API, Telegram or a TradingView watchlist.
 Is that a question your support team or user groups hear often?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1078,7 +1078,7 @@
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy; email from domain-restricted search snippet. City inferred from 02 area code (Sydney). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy; email from domain-restricted search snippet. City inferred from 02 area code (Sydney). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For CMC Connect partners that usually means custom trading bots and integration scripts built against the platform they license.
 Is there a CMC Connect contact who handles partner developer questions?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1200,7 +1200,7 @@
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. UK-listed group; Australian entity and office clearly shown. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. UK-listed group; Australian entity and office clearly shown. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For FP Markets that could mean a referral developer for clients who want custom EAs, indicators or cTrader cBots.
 Would your team be open to hearing how that referral could work?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1323,7 +1323,7 @@
       <c r="W7" s="3" t="n"/>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For you that could mean building client-side bots and scripts on the IR API, or internal tools for the OTC workflow.
 Who would be the right person to talk to about developer support for API clients?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1448,7 +1448,7 @@
       <c r="W8" s="3" t="n"/>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Sydney) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Sydney) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a broker like IC Markets that usually means a dependable developer you can point clients to for EA builds and MQL-to-cBot conversions.
 Would your partnerships team be open to a short conversation about that?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1570,7 +1570,7 @@
       <c r="W9" s="3" t="n"/>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Vantage that could mean converting client Pine Script strategies into MT4/MT5 EAs, or building bots for copy trading signal providers.
 Would it be useful to have a developer your team can refer those requests to?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1693,7 +1693,7 @@
       <c r="W10" s="3" t="n"/>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Vantage group operates globally; AU office confirmed by address in results. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Vantage group operates globally; AU office confirmed by address in results. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
 For a quant equity team, the relevant part is usually contained Python tooling: data loaders, backtest utilities or order file generation that plugs into your existing process.
 Does your team ever bring in outside developers for that sort of side tooling?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1818,7 +1818,7 @@
       <c r="W11" s="3" t="n"/>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Client-team (investor relations) inbox; institutional manager, outsourcing likelihood modest. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Client-team (investor relations) inbox; institutional manager, outsourcing likelihood modest. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
 For a desk like yours that usually means taking one of those side projects, such as a new venue connector or a research backtest tool, and delivering it as a contained piece of work your engineers can review.
 Is outside help on non-core trading tooling something your commercial team ever considers?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -1942,7 +1942,7 @@
       <c r="W12" s="3" t="n"/>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Alternative: commercial@vivcourt.com for trading-related enquiries. Large sophisticated firm; low likelihood of outsourcing core systems. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Alternative: commercial@vivcourt.com for trading-related enquiries. Large sophisticated firm; low likelihood of outsourcing core systems. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2025,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For an agency like yours that usually means white-label help on the platform-specific pieces while you keep the client relationship.
 Would it be useful to have a specialist you can hand those platform-specific jobs to?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2065,7 +2065,7 @@
       <c r="W13" s="3" t="n"/>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Digital Surge that would mean building rule-based bots or partner integrations on top of those endpoints.
 Would you be open to a quick chat about developers building on your API?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2190,7 +2190,7 @@
       <c r="W14" s="3" t="n"/>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Brisbane) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Brisbane) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a screening service like yours, the useful piece is often a connector that sends screen hits to alerts or a broker API rather than a full trading bot.
 Have subscribers asked for anything along those lines?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2313,7 +2313,7 @@
       <c r="W15" s="3" t="n"/>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy. City inferred from 07 5632 number (Gold Coast region); reviewer should confirm. Email association from snippet only. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy. City inferred from 07 5632 number (Gold Coast region); reviewer should confirm. Email association from snippet only. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2396,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a charting vendor like Optuma that could mean acting as an outside developer you refer clients to when they want signals executed on MT5, TradingView or a broker API.
 Do you ever get consultation requests that go beyond what Optuma scripting covers?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2436,7 +2436,7 @@
       <c r="W16" s="3" t="n"/>
       <c r="X16" s="2" t="inlineStr">
         <is>
-          <t>Egress to optuma.com blocked from this environment; email seen in domain-restricted search snippet for the contact page, not opened directly. Market Analyst is the former name of Optuma, so treated as the same company. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Egress to optuma.com blocked from this environment; email seen in domain-restricted search snippet for the contact page, not opened directly. Market Analyst is the former name of Optuma, so treated as the same company. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For an exchange like yours that could mean reference bots or integration builds for API clients, or internal tooling around order execution.
 Is there anyone on the partnerships or institutional side who looks at third-party developers working with the API?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2561,7 +2561,7 @@
       <c r="W17" s="3" t="n"/>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2650,7 @@
 For a strategy-subscription business like yours, that usually means converting existing system rules into scheduled scanners, order-generation scripts or broker-connected execution, with logs members can audit.
 Is automating any part of the member signal or execution workflow something you have looked at recently?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2690,7 +2690,7 @@
       <c r="W18" s="3" t="n"/>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>WebFetch was egress-blocked for this domain, so email seen via search result from the prospect's own bio PDF (dated 2014) only - verify still active before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch was egress-blocked for this domain, so email seen via search result from the prospect's own bio PDF (dated 2014) only - verify still active before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a studio like yours that usually means a contractor who can pick up the MQL or Pine side of a project under your brand.
 Is that kind of cross-platform request something you currently turn away or build in-house?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2813,7 +2813,7 @@
       <c r="W19" s="3" t="n"/>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Two different Adelaide addresses appear in snippets. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Two different Adelaide addresses appear in snippets. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
 For a hybrid like yours, that could be automated balance and drawdown monitoring, payout reconciliation scripts, or trade-management tools for subscribers.
 Who on your team looks after the trading-platform side of things?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -2938,7 +2938,7 @@
       <c r="W20" s="3" t="n"/>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>WebFetch and direct HTTP were blocked by the network egress proxy for every site in this session, and the shared WebSearch budget ran out partway through. The email and facts come from search results that cite the prospect's own pages. Open the source page to confirm before sending. The site says its services are not currently for Australian residents (they have a waitlist), but the business is based in Australia. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch and direct HTTP were blocked by the network egress proxy for every site in this session, and the shared WebSearch budget ran out partway through. The email and facts come from search results that cite the prospect's own pages. Open the source page to confirm before sending. The site says its services are not currently for Australian residents (they have a waitlist), but the business is based in Australia. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. Here that mostly means porting or rebuilding client bots and order-management scripts on API v3.
 Would it be useful to have a developer you can refer API clients to when they ask for help?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3063,7 +3063,7 @@
       <c r="W21" s="3" t="n"/>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3146,7 +3146,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Beyond Charts that could be an MT5 or TradingView version of the methodology signals for CFD users, built as an add-on.
 Is porting the methodology to other platforms something you have considered?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3187,7 +3187,7 @@
       <c r="W22" s="3" t="n"/>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy; city inferred from 03 9583 number (Melbourne south-east). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy; city inferred from 03 9583 number (Melbourne south-east). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. With CoinJar that would mostly be strategy bots and order logic built on the Trading API, using trade-scoped keys only.
 Is referring API clients to outside developers something your team does?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3312,7 +3312,7 @@
       <c r="W23" s="3" t="n"/>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Eightcap that would mean a developer who picks up where Capitalise.ai stops: custom MT4/MT5 EAs and Pine Script alert systems.
 Does your team see clients asking for more than the no-code tools cover?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3435,7 +3435,7 @@
       <c r="W24" s="3" t="n"/>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. global@eightcap.com also listed as an alternative. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. global@eightcap.com also listed as an alternative. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3518,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Fusion that could mean a developer your Master traders can use to automate and stress-test the strategies they publish on Fusion+.
 Who on your side looks after Fusion+ Master traders?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3560,7 +3560,7 @@
       <c r="W25" s="3" t="n"/>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For GO Markets that might mean building bespoke EAs or indicators for clients, or extra utilities that sit alongside Genesis.
 Is that kind of client request something your platform team ever receives?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3682,7 +3682,7 @@
       <c r="W26" s="3" t="n"/>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3765,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a vendor of Iress's size, the fit is probably as a contractor for client-specific integrations rather than platform work.
 Is there a partner or integrations contact I should speak with instead?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3805,7 +3805,7 @@
       <c r="W27" s="3" t="n"/>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>Large enterprise; low likelihood of buying but qualified. Email from domain-restricted snippet; exact page not confirmed. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Large enterprise; low likelihood of buying but qualified. Email from domain-restricted snippet; exact page not confirmed. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For an API provider, I could be a developer your partners are pointed to for strategy execution and order-management builds against the Openmarkets API.
 Would a referral arrangement like that be of interest to your API team?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -3928,7 +3928,7 @@
       <c r="W28" s="3" t="n"/>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy. City (Melbourne) from general knowledge, not re-verified in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy. City (Melbourne) from general knowledge, not re-verified in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Pepperstone that would mean acting as a referral developer who converts client strategies into EAs or C# cBots that run cleanly on your servers.
 Is there a partner or IB contact who looks after developer referrals I could speak with?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4052,7 +4052,7 @@
       <c r="W29" s="3" t="n"/>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a broker like yours that usually means someone who can build client-side connectors and rule-based execution scripts against the platform.
 Who on your side handles those API integration requests, and would a developer referral be useful to them?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4174,7 +4174,7 @@
       <c r="W30" s="3" t="n"/>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Perth office alternative: advice@phillipsecurities.com.au. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Perth office alternative: advice@phillipsecurities.com.au. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
 For a mechanical-system vendor, that typically means broker-connected order routing, alerting, or a backtest harness that sits alongside your existing software.
 Would it be useful to compare notes on how SPA3 subscribers currently get from a signal to a placed trade?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4304,7 +4304,7 @@
       <c r="W31" s="3" t="n"/>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>WebFetch egress-blocked; email seen in domain-restricted search result only (exact page not pinpointed - likely home/privacy page). Cheltenham location came from a third-party directory summary. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch egress-blocked; email seen in domain-restricted search result only (exact page not pinpointed - likely home/privacy page). Cheltenham location came from a third-party directory summary. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For ThinkMarkets that would mean a developer who builds and backtests EAs for clients before they move them onto your VPS.
 Is there someone in partnerships I should send a short intro to?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4427,7 +4427,7 @@
       <c r="W32" s="3" t="n"/>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
 For a crypto liquidity business that usually means exchange API connectors, automated hedging scripts or monitoring that flags stale quotes before a client does.
 Would it be useful to talk through any exchange integrations sitting in your backlog?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4553,7 +4553,7 @@
       <c r="W33" s="3" t="n"/>
       <c r="X33" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact page carrying hello@zerocap.com not isolated among zerocap.com pages returned (contact, services, about); media@zerocap.com also mentioned. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact page carrying hello@zerocap.com not isolated among zerocap.com pages returned (contact, services, about); media@zerocap.com also mentioned. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4636,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For ACY that might mean overflow development: EAs, indicators or bridge scripts for clients and IBs.
 Who would be the right person to talk to about outside development capacity?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4675,7 +4675,7 @@
       <c r="W34" s="3" t="n"/>
       <c r="X34" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Specific technology products not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Specific technology products not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For Global Prime that would mean a developer you can refer clients to for bespoke EAs built around ECN execution.
 Is that a request your support desk ever hears?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4798,7 +4798,7 @@
       <c r="W35" s="3" t="n"/>
       <c r="X35" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Platform offering not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Platform offering not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
 I build custom trading bots and automation systems for platforms such as MT4, MT5, TradingView and crypto exchanges. For a firm like yours that usually means a subcontractor for the strategy and execution layer while your team handles the platform and front end.
 Would you consider bringing in outside help on the bot logic for upcoming projects?
 Best regards,
-[Your Name]
+Gabriel
 goodfiberr@gmail.com</t>
         </is>
       </c>
@@ -4920,7 +4920,7 @@
       <c r="W36" s="3" t="n"/>
       <c r="X36" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Snippet did not clearly identify which page carried the email; confirm on contact page. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace [Your Name] in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Snippet did not clearly identify which page carried the email; confirm on contact page. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop obsolete sender-name note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAWtfhwVbimX9RKznBAhMh
</commit_message>
<xml_diff>
--- a/Australia_Trading_Bot_Prospects_200.xlsx
+++ b/Australia_Trading_Bot_Prospects_200.xlsx
@@ -701,7 +701,7 @@
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. State/city not verified this session (search budget exhausted); fill in before use. QC: state '' not an Australian state/territory; email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. State/city not verified this session (search budget exhausted); fill in before use. QC: state '' not an Australian state/territory; email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact apollocrypto.com page carrying the email not isolated (funds/wholesale/home pages returned). Sydney location from general knowledge, not re-verified this session. Strategy is largely discretionary/fundamental, not purely systematic. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact apollocrypto.com page carrying the email not isolated (funds/wholesale/home pages returned). Sydney location from general knowledge, not re-verified this session. Strategy is largely discretionary/fundamental, not purely systematic. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       <c r="W4" s="3" t="n"/>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy; email from domain-restricted search snippet. City inferred from 02 area code (Sydney). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy; email from domain-restricted search snippet. City inferred from 02 area code (Sydney). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. UK-listed group; Australian entity and office clearly shown. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. UK-listed group; Australian entity and office clearly shown. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
       <c r="W7" s="3" t="n"/>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       <c r="W8" s="3" t="n"/>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Sydney) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Sydney) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1570,7 @@
       <c r="W9" s="3" t="n"/>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       <c r="W10" s="3" t="n"/>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Vantage group operates globally; AU office confirmed by address in results. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Vantage group operates globally; AU office confirmed by address in results. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       <c r="W11" s="3" t="n"/>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Client-team (investor relations) inbox; institutional manager, outsourcing likelihood modest. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Client-team (investor relations) inbox; institutional manager, outsourcing likelihood modest. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       <c r="W12" s="3" t="n"/>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Alternative: commercial@vivcourt.com for trading-related enquiries. Large sophisticated firm; low likelihood of outsourcing core systems. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Alternative: commercial@vivcourt.com for trading-related enquiries. Large sophisticated firm; low likelihood of outsourcing core systems. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       <c r="W13" s="3" t="n"/>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       <c r="W14" s="3" t="n"/>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Brisbane) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Brisbane) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       <c r="W15" s="3" t="n"/>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy. City inferred from 07 5632 number (Gold Coast region); reviewer should confirm. Email association from snippet only. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy. City inferred from 07 5632 number (Gold Coast region); reviewer should confirm. Email association from snippet only. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       <c r="W16" s="3" t="n"/>
       <c r="X16" s="2" t="inlineStr">
         <is>
-          <t>Egress to optuma.com blocked from this environment; email seen in domain-restricted search snippet for the contact page, not opened directly. Market Analyst is the former name of Optuma, so treated as the same company. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Egress to optuma.com blocked from this environment; email seen in domain-restricted search snippet for the contact page, not opened directly. Market Analyst is the former name of Optuma, so treated as the same company. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       <c r="W17" s="3" t="n"/>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       <c r="W18" s="3" t="n"/>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>WebFetch was egress-blocked for this domain, so email seen via search result from the prospect's own bio PDF (dated 2014) only - verify still active before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch was egress-blocked for this domain, so email seen via search result from the prospect's own bio PDF (dated 2014) only - verify still active before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       <c r="W19" s="3" t="n"/>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Two different Adelaide addresses appear in snippets. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Two different Adelaide addresses appear in snippets. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       <c r="W20" s="3" t="n"/>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>WebFetch and direct HTTP were blocked by the network egress proxy for every site in this session, and the shared WebSearch budget ran out partway through. The email and facts come from search results that cite the prospect's own pages. Open the source page to confirm before sending. The site says its services are not currently for Australian residents (they have a waitlist), but the business is based in Australia. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch and direct HTTP were blocked by the network egress proxy for every site in this session, and the shared WebSearch budget ran out partway through. The email and facts come from search results that cite the prospect's own pages. Open the source page to confirm before sending. The site says its services are not currently for Australian residents (they have a waitlist), but the business is based in Australia. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       <c r="W21" s="3" t="n"/>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       <c r="W22" s="3" t="n"/>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy; city inferred from 03 9583 number (Melbourne south-east). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy; city inferred from 03 9583 number (Melbourne south-east). QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       <c r="W23" s="3" t="n"/>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Direct site fetch (WebFetch/curl) was blocked by the session egress proxy for every exchange domain; email seen in a web-search result restricted to/attributed to the company's own domain, not on a page opened directly. Re-verify before sending. City (Melbourne) from general knowledge, not re-confirmed in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       <c r="W24" s="3" t="n"/>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. global@eightcap.com also listed as an alternative. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. global@eightcap.com also listed as an alternative. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3560,7 @@
       <c r="W25" s="3" t="n"/>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3682,7 @@
       <c r="W26" s="3" t="n"/>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
       <c r="W27" s="3" t="n"/>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>Large enterprise; low likelihood of buying but qualified. Email from domain-restricted snippet; exact page not confirmed. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Large enterprise; low likelihood of buying but qualified. Email from domain-restricted snippet; exact page not confirmed. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
       <c r="W28" s="3" t="n"/>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>Site blocked by egress proxy. City (Melbourne) from general knowledge, not re-verified in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Site blocked by egress proxy. City (Melbourne) from general knowledge, not re-verified in this session. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       <c r="W29" s="3" t="n"/>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       <c r="W30" s="3" t="n"/>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Perth office alternative: advice@phillipsecurities.com.au. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Perth office alternative: advice@phillipsecurities.com.au. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       <c r="W31" s="3" t="n"/>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>WebFetch egress-blocked; email seen in domain-restricted search result only (exact page not pinpointed - likely home/privacy page). Cheltenham location came from a third-party directory summary. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch egress-blocked; email seen in domain-restricted search result only (exact page not pinpointed - likely home/privacy page). Cheltenham location came from a third-party directory summary. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
       <c r="W32" s="3" t="n"/>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4553,7 @@
       <c r="W33" s="3" t="n"/>
       <c r="X33" s="2" t="inlineStr">
         <is>
-          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact page carrying hello@zerocap.com not isolated among zerocap.com pages returned (contact, services, about); media@zerocap.com also mentioned. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>Email seen in web search result drawn from the prospect's own domain only; WebFetch was blocked by the session egress proxy so the page could not be opened directly. Reviewer should open source_url to confirm before sending. Exact page carrying hello@zerocap.com not isolated among zerocap.com pages returned (contact, services, about); media@zerocap.com also mentioned. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4675,7 @@
       <c r="W34" s="3" t="n"/>
       <c r="X34" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Specific technology products not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Specific technology products not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4798,7 +4798,7 @@
       <c r="W35" s="3" t="n"/>
       <c r="X35" s="2" t="inlineStr">
         <is>
-          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Platform offering not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch to the company domain was blocked by the network egress proxy in this environment; email seen in full in search results attributed to the company's own contact page (not opened directly). Re-verify on the live page before sending. Platform offering not re-verified because the search budget ran out. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
       <c r="W36" s="3" t="n"/>
       <c r="X36" s="2" t="inlineStr">
         <is>
-          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Snippet did not clearly identify which page carried the email; confirm on contact page. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending Replace the sender name in the sign-off before sending.</t>
+          <t>WebFetch/curl to this domain was blocked by the session egress proxy; email seen in full in a search-result snippet attributed to the company's own domain, consistent with that domain. Re-verify on the live page before sending. Snippet did not clearly identify which page carried the email; confirm on contact page. QC: email seen in search results only - source page could not be opened this session; confirm it on the live page before sending</t>
         </is>
       </c>
     </row>

</xml_diff>